<commit_message>
Conciliación: biblias verificadas, el grupo pagó las 52
El reembolso a JM del 19/08 es 35,360 = 52 × 680 exactos. El presupuesto
oficial solo contemplaba 50 (34,000) porque 2 las pagaría Camila
Fernández: esas 2 (1,360) quedaron dentro de lo que pagó el grupo. No hay
aporte suyo en las 49 donaciones ni ningún movimiento de 1,360.

Queda por confirmar con ella si puso el dinero de su bolsillo, para
reembolsarlo o registrarlo como donación en especie. La caja y el cuadre
con el banco no cambian en ningún caso.

Auditoría: 37/37. verify.py: 9/9 PASS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016scja59CycFFrqKgYsUPWh
</commit_message>
<xml_diff>
--- a/data/presupuesto/Conciliacion_Final_ETC88.xlsx
+++ b/data/presupuesto/Conciliacion_Final_ETC88.xlsx
@@ -803,7 +803,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3816000" cy="2951999"/>
@@ -825,7 +825,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3816000" cy="2951999"/>
@@ -1136,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1502,7 +1502,7 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>PENDIENTES (0 abiertos · 1 notas)</t>
+          <t>PENDIENTES (0 abiertos · 2 notas)</t>
         </is>
       </c>
     </row>
@@ -1518,142 +1518,154 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Biblias: las 2 de Camila</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Confirmar con Camila y con Juan Manuel: si ella puso 1,360 de su bolsillo, o se le reembolsa, o se registra como donación en especie (el costo del retiro subiría a 618,429 y la especie a 93,765). La caja y el cuadre con el banco no cambian en ningún caso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>DISTRIBUCIÓN DEL DINERO</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Izquierda: de dónde salió cada peso que entró. Derecha: en qué se fue cada peso que salió de caja.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>HOJAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>1 Caja</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="inlineStr">
-        <is>
-          <t>entradas por fuente, salidas, balance, banco</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
-          <t>2 Presupuesto vs costo</t>
+          <t>1 Caja</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>presupuestado → costó → cubierto sin pagar → pagado de caja, por área</t>
+          <t>entradas por fuente, salidas, balance, banco</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>3 Al costo vs caja</t>
+          <t>2 Presupuesto vs costo</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>qué vale el retiro y qué nos costó; la casa al detalle</t>
+          <t>presupuestado → costó → cubierto sin pagar → pagado de caja, por área</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="inlineStr">
         <is>
-          <t>4 Base ETC 89</t>
+          <t>3 Al costo vs caja</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>costo real por partida y por persona; recomendaciones para el próximo</t>
+          <t>qué vale el retiro y qué nos costó; la casa al detalle</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
         <is>
-          <t>5 Pendientes</t>
+          <t>4 Base ETC 89</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>una sola lista: abiertos, notas, cerrados</t>
+          <t>costo real por partida y por persona; recomendaciones para el próximo</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="15" t="inlineStr">
         <is>
-          <t>6 Ppto oficial vs Sistem</t>
+          <t>5 Pendientes</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>los dos presupuestos por área</t>
+          <t>una sola lista: abiertos, notas, cerrados</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="inlineStr">
         <is>
-          <t>7–10 Anexos</t>
+          <t>6 Ppto oficial vs Sistem</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Gastos · Donaciones efectivo · Especie · Profondo (con la liquidación de la comisión)</t>
+          <t>los dos presupuestos por área</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>11 Auditoría</t>
+          <t>7–10 Anexos</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>36 verificaciones recalculadas (36 cuadran)</t>
+          <t>Gastos · Donaciones efectivo · Especie · Profondo (con la liquidación de la comisión)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>12 Fuentes y método</t>
+          <t>11 Auditoría</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>de dónde sale cada número y las reglas usadas</t>
+          <t>37 verificaciones recalculadas (37 cuadran)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
+          <t>12 Fuentes y método</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>de dónde sale cada número y las reglas usadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
           <t>13 Notas por partida</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>la explicación de cada partida del presupuesto</t>
         </is>
@@ -2594,7 +2606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3473,14 +3485,14 @@
       </c>
       <c r="B36" s="39" t="inlineStr">
         <is>
-          <t>Biblias: reembolso 35,360 = proforma 34,000 + 1,360; donaciones etiquetadas "biblia"</t>
+          <t>Biblias: el pago de 35,360 = 52 × 680 exactos</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>16500</v>
+        <v>35360</v>
       </c>
       <c r="D36" s="17" t="n">
-        <v>16500</v>
+        <v>35360</v>
       </c>
       <c r="E36" s="86" t="inlineStr">
         <is>
@@ -3489,7 +3501,7 @@
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>Roosbert, Pamela Nivar, Carol, Kharla, Wirna</t>
+          <t>el presupuesto tenía 50 (34,000); las 2 de más (1,360) son las que iba a pagar Camila</t>
         </is>
       </c>
     </row>
@@ -3499,14 +3511,14 @@
       </c>
       <c r="B37" s="39" t="inlineStr">
         <is>
-          <t>Donaciones que requieren nota: el depósito sin dueño y la de Yendry sin captura</t>
+          <t>Biblias: donaciones en efectivo etiquetadas "biblia"</t>
         </is>
       </c>
       <c r="C37" s="17" t="n">
-        <v>2000</v>
+        <v>16500</v>
       </c>
       <c r="D37" s="17" t="n">
-        <v>2000</v>
+        <v>16500</v>
       </c>
       <c r="E37" s="86" t="inlineStr">
         <is>
@@ -3515,7 +3527,7 @@
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
-          <t>las de Wilfrid y Johan se ubicaron: ya no llevan nota</t>
+          <t>Roosbert, Pamela Nivar, Carol, Kharla, Wirna</t>
         </is>
       </c>
     </row>
@@ -3525,21 +3537,25 @@
       </c>
       <c r="B38" s="39" t="inlineStr">
         <is>
-          <t>Costo del retiro = caja + especie + cortesías (8 × 500 + 2 × 2,360)</t>
+          <t>Donaciones que requieren nota: el depósito sin dueño y la de Yendry sin captura</t>
         </is>
       </c>
       <c r="C38" s="17" t="n">
-        <v>617069</v>
+        <v>2000</v>
       </c>
       <c r="D38" s="17" t="n">
-        <v>617069</v>
+        <v>2000</v>
       </c>
       <c r="E38" s="86" t="inlineStr">
         <is>
           <t>Cuadra</t>
         </is>
       </c>
-      <c r="F38" s="18" t="inlineStr"/>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>las de Wilfrid y Johan se ubicaron: ya no llevan nota</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="85" t="n">
@@ -3547,26 +3563,48 @@
       </c>
       <c r="B39" s="39" t="inlineStr">
         <is>
+          <t>Costo del retiro = caja + especie + cortesías (8 × 500 + 2 × 2,360)</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="n">
+        <v>617069</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <v>617069</v>
+      </c>
+      <c r="E39" s="86" t="inlineStr">
+        <is>
+          <t>Cuadra</t>
+        </is>
+      </c>
+      <c r="F39" s="18" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="85" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="39" t="inlineStr">
+        <is>
           <t>Apoyo total donado = efectivo + especie</t>
         </is>
       </c>
-      <c r="C39" s="17" t="n">
+      <c r="C40" s="17" t="n">
         <v>247426</v>
       </c>
-      <c r="D39" s="17" t="n">
+      <c r="D40" s="17" t="n">
         <v>247426</v>
       </c>
-      <c r="E39" s="86" t="inlineStr">
+      <c r="E40" s="86" t="inlineStr">
         <is>
           <t>Cuadra</t>
         </is>
       </c>
-      <c r="F39" s="18" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>36 de 36 verificaciones cuadran</t>
+      <c r="F40" s="18" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>37 de 37 verificaciones cuadran</t>
         </is>
       </c>
     </row>
@@ -4062,12 +4100,12 @@
       </c>
       <c r="B12" s="39" t="inlineStr">
         <is>
-          <t>Biblias (50 × 680)</t>
+          <t>Biblias (52 × 680)</t>
         </is>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>Reembolso a JM (19/08): proforma Paulinas 34,000 + 1,360. Donaciones en efectivo etiquetadas "biblia": 16,500</t>
+          <t>Se pidieron 52 y el grupo pagó las 52: 52 × 680 = 35,360 exactos (reembolso a JM, 19/08). El presupuesto oficial solo contemplaba 50 (34,000) porque 2 las pagaría Camila; esas 2 (1,360) quedaron dentro de lo que pagó el grupo. Financiadas en parte por 16,500 de donaciones en efectivo etiquetadas "biblia"</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5130,7 @@
     <row r="15" outlineLevel="1">
       <c r="B15" s="39" t="inlineStr">
         <is>
-          <t>Biblias (50 × 680)</t>
+          <t>Biblias (52 × 680)</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
@@ -6580,7 +6618,7 @@
       </c>
       <c r="B12" s="39" t="inlineStr">
         <is>
-          <t>Biblias (50 × 680)</t>
+          <t>Biblias (52 × 680)</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
@@ -7585,7 +7623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7747,22 +7785,26 @@
       <c r="D9" s="18" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="69" t="inlineStr">
-        <is>
-          <t>CERRADO</t>
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>NOTA</t>
         </is>
       </c>
       <c r="B10" s="70" t="inlineStr">
         <is>
-          <t>Impresión de libretas 1,260</t>
+          <t>Biblias: las 2 de Camila</t>
         </is>
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
-          <t>El presupuesto operativo la marcaba "donado por guías" en la columna equivocada, por eso no sumaba. Sumada a la especie por confirmación del director (11-sep).</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr"/>
+          <t>Se pidieron 52 biblias y el grupo pagó las 52: el reembolso a JM del 19/08 es 35,360 = 52 × 680 exactos. El presupuesto solo contemplaba 50 (34,000) porque 2 las pagaría Camila Fernández; esas 2 quedaron dentro de lo que pagó el grupo. En las 49 donaciones en efectivo no hay ningún aporte suyo ni ningún movimiento de 1,360, y en la especie solo figura por los separadores de libros (750).</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar con Camila y con Juan Manuel: si ella puso 1,360 de su bolsillo, o se le reembolsa, o se registra como donación en especie (el costo del retiro subiría a 618,429 y la especie a 93,765). La caja y el cuadre con el banco no cambian en ningún caso.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="69" t="inlineStr">
@@ -7772,12 +7814,12 @@
       </c>
       <c r="B11" s="70" t="inlineStr">
         <is>
-          <t>Uso de los 34,337 en cuentas</t>
+          <t>Impresión de libretas 1,260</t>
         </is>
       </c>
       <c r="C11" s="39" t="inlineStr">
         <is>
-          <t>La dirección lo expondrá en la actividad de cierre (evaluación) del ETC 88 para decidirlo con el equipo (11-sep).</t>
+          <t>El presupuesto operativo la marcaba "donado por guías" en la columna equivocada, por eso no sumaba. Sumada a la especie por confirmación del director (11-sep).</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr"/>
@@ -7790,12 +7832,12 @@
       </c>
       <c r="B12" s="70" t="inlineStr">
         <is>
-          <t>Profondo: liquidación de la comisión</t>
+          <t>Uso de los 34,337 en cuentas</t>
         </is>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>Bruto 154,420: 680.5 boletas pagadas × 200 = 136,100 + venta de comida y helados 18,320. Premios 19,900 (aire acondicionado 16,900 + abanico de torre 3,000). Neto del informe 134,520; entregado a finanzas 135,866.40: los 1,346.40 adicionales son ventas de helados posteriores al informe (director).</t>
+          <t>La dirección lo expondrá en la actividad de cierre (evaluación) del ETC 88 para decidirlo con el equipo (11-sep).</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr"/>
@@ -7808,12 +7850,12 @@
       </c>
       <c r="B13" s="70" t="inlineStr">
         <is>
-          <t>Pagaron y no fueron</t>
+          <t>Profondo: liquidación de la comisión</t>
         </is>
       </c>
       <c r="C13" s="39" t="inlineStr">
         <is>
-          <t>Verificado nombre por nombre contra la lista de pagos del director (10-sep, 57 líneas), el registro de cuotas y las 49 donaciones. Equipo: Mary Carmen Ramírez pagó y no asistió; sus 2,000 están dentro de los 98,000. Participantes: los 46 que pagaron están todos identificados con nombre y ninguno figura como ausente. Boris pagó, no fue, se le devolvió una parte y el neto de 1,500 entró como donación a nombre de Jonathan Medina (31/08): su dinero NO está en los 156,800. De Amanda Rivera no hay ningún pago en ninguna fuente; solo aparece en el formulario de junio como invitada de Pamela Colón y Roselyn Quiroz. Los únicos abonos de 500 de la lista son de Melany Ceverino y Erilis Polanco, ambas personas que sí asistieron.</t>
+          <t>Bruto 154,420: 680.5 boletas pagadas × 200 = 136,100 + venta de comida y helados 18,320. Premios 19,900 (aire acondicionado 16,900 + abanico de torre 3,000). Neto del informe 134,520; entregado a finanzas 135,866.40: los 1,346.40 adicionales son ventas de helados posteriores al informe (director).</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr"/>
@@ -7826,12 +7868,12 @@
       </c>
       <c r="B14" s="70" t="inlineStr">
         <is>
-          <t>Presupuesto oficial</t>
+          <t>Pagaron y no fueron</t>
         </is>
       </c>
       <c r="C14" s="39" t="inlineStr">
         <is>
-          <t>Declarado OFICIAL el de 11-Ago (596,249.56, costo completo, tarifa real de la casa). El Sistem (512,859.56) es la referencia operativa del tablero.</t>
+          <t>Verificado nombre por nombre contra la lista de pagos del director (10-sep, 57 líneas), el registro de cuotas y las 49 donaciones. Equipo: Mary Carmen Ramírez pagó y no asistió; sus 2,000 están dentro de los 98,000. Participantes: los 46 que pagaron están todos identificados con nombre y ninguno figura como ausente. Boris pagó, no fue, se le devolvió una parte y el neto de 1,500 entró como donación a nombre de Jonathan Medina (31/08): su dinero NO está en los 156,800. De Amanda Rivera no hay ningún pago en ninguna fuente; solo aparece en el formulario de junio como invitada de Pamela Colón y Roselyn Quiroz. Los únicos abonos de 500 de la lista son de Melany Ceverino y Erilis Polanco, ambas personas que sí asistieron.</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr"/>
@@ -7844,19 +7886,15 @@
       </c>
       <c r="B15" s="70" t="inlineStr">
         <is>
-          <t>Pago a JM 37,500</t>
+          <t>Presupuesto oficial</t>
         </is>
       </c>
       <c r="C15" s="39" t="inlineStr">
         <is>
-          <t>Desglosado en la hoja de Gastos: transporte 2ª mitad 17,500 (10,000 + 7,500) + desvío 10,000 + ofrenda P. Héctor 10,000.</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Registrar el desglose en el tablero.</t>
-        </is>
-      </c>
+          <t>Declarado OFICIAL el de 11-Ago (596,249.56, costo completo, tarifa real de la casa). El Sistem (512,859.56) es la referencia operativa del tablero.</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="69" t="inlineStr">
@@ -7866,15 +7904,19 @@
       </c>
       <c r="B16" s="70" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Pago a JM 37,500</t>
         </is>
       </c>
       <c r="C16" s="39" t="inlineStr">
         <is>
-          <t>Fuimos 99, facturadas 97. Cortesías: el padre y la sor (la del director cedida a la sor). Jueves: 27 personas, 19 pagaron 500, 8 sin cobro. Habitaciones de pequeños grupos: 900 × 2 noches. Total 240,220 = avance 23,600 + final 216,620.</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr"/>
+          <t>Desglosado en la hoja de Gastos: transporte 2ª mitad 17,500 (10,000 + 7,500) + desvío 10,000 + ofrenda P. Héctor 10,000.</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Registrar el desglose en el tablero.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="69" t="inlineStr">
@@ -7884,12 +7926,12 @@
       </c>
       <c r="B17" s="70" t="inlineStr">
         <is>
-          <t>Bizcocho y helados</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="C17" s="39" t="inlineStr">
         <is>
-          <t>Bizcocho de bienvenida 6,000 (10/09, no presupuestado). El bizcocho de la dinámica (ppto Cocina 1,500) se cambió por helados: 1,740 (07/09). La venta de helados del profondo es ingreso, no costo.</t>
+          <t>Fuimos 99, facturadas 97. Cortesías: el padre y la sor (la del director cedida a la sor). Jueves: 27 personas, 19 pagaron 500, 8 sin cobro. Habitaciones de pequeños grupos: 900 × 2 noches. Total 240,220 = avance 23,600 + final 216,620.</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr"/>
@@ -7902,12 +7944,12 @@
       </c>
       <c r="B18" s="70" t="inlineStr">
         <is>
-          <t>Lapiceros e insumos de misa</t>
+          <t>Bizcocho y helados</t>
         </is>
       </c>
       <c r="C18" s="39" t="inlineStr">
         <is>
-          <t>Caja de lapiceros (650) donada; insumos de misa (3,000) asumidos por Jonathan Medina y Fernando Cordero. Ambos en la especie.</t>
+          <t>Bizcocho de bienvenida 6,000 (10/09, no presupuestado). El bizcocho de la dinámica (ppto Cocina 1,500) se cambió por helados: 1,740 (07/09). La venta de helados del profondo es ingreso, no costo.</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr"/>
@@ -7920,12 +7962,12 @@
       </c>
       <c r="B19" s="70" t="inlineStr">
         <is>
-          <t>Impresiones de guías</t>
+          <t>Lapiceros e insumos de misa</t>
         </is>
       </c>
       <c r="C19" s="39" t="inlineStr">
         <is>
-          <t>Mochilas (3,600, pagadas) e "impresiones diversas" (3,600, donadas por Darianny) son trabajos distintos. No hay doble conteo.</t>
+          <t>Caja de lapiceros (650) donada; insumos de misa (3,000) asumidos por Jonathan Medina y Fernando Cordero. Ambos en la especie.</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr"/>
@@ -7938,12 +7980,12 @@
       </c>
       <c r="B20" s="70" t="inlineStr">
         <is>
-          <t>Priscila</t>
+          <t>Impresiones de guías</t>
         </is>
       </c>
       <c r="C20" s="39" t="inlineStr">
         <is>
-          <t>Donó materiales (7,340) y recibió 2,000 en efectivo (21/07). Donación neta 5,340; la especie ya lo descuenta.</t>
+          <t>Mochilas (3,600, pagadas) e "impresiones diversas" (3,600, donadas por Darianny) son trabajos distintos. No hay doble conteo.</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr"/>
@@ -7956,37 +7998,37 @@
       </c>
       <c r="B21" s="70" t="inlineStr">
         <is>
+          <t>Priscila</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>Donó materiales (7,340) y recibió 2,000 en efectivo (21/07). Donación neta 5,340; la especie ya lo descuenta.</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="69" t="inlineStr">
+        <is>
+          <t>CERRADO</t>
+        </is>
+      </c>
+      <c r="B22" s="70" t="inlineStr">
+        <is>
           <t>Balance 117,611 de la hoja General</t>
         </is>
       </c>
-      <c r="C21" s="39" t="inlineStr">
+      <c r="C22" s="39" t="inlineStr">
         <is>
           <t>Cifra escrita a mano hacia el 11-ago, antes del retiro. No es un segundo balance. El oficial es 36,543.40 → real 34,337.</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Borrar o anotar esa cifra en la hoja de presupuesto.</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="71" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="B22" s="70" t="inlineStr">
-        <is>
-          <t>Especie</t>
-        </is>
-      </c>
-      <c r="C22" s="39" t="inlineStr">
-        <is>
-          <t>Total 92,405: la hoja de presupuesto solo tenía marcados 30,301 (marcas sin actualizar). Peces (36,000), decoración (10,300), Bono Olé (4,588), insumos de misa (3,000), oficina, lapiceros y cocina no estaban marcados.</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="71" t="inlineStr">
@@ -7996,12 +8038,12 @@
       </c>
       <c r="B23" s="70" t="inlineStr">
         <is>
-          <t>Oficina</t>
+          <t>Especie</t>
         </is>
       </c>
       <c r="C23" s="39" t="inlineStr">
         <is>
-          <t>Costo real 5,306.11 asumido por los directores; en la especie se valora a ppto (2,300) por instrucción del director. Solo informativo.</t>
+          <t>Total 92,405: la hoja de presupuesto solo tenía marcados 30,301 (marcas sin actualizar). Peces (36,000), decoración (10,300), Bono Olé (4,588), insumos de misa (3,000), oficina, lapiceros y cocina no estaban marcados.</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr"/>
@@ -8014,12 +8056,12 @@
       </c>
       <c r="B24" s="70" t="inlineStr">
         <is>
-          <t>Presupuestos "Tentativo"</t>
+          <t>Oficina</t>
         </is>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
-          <t>Ambos quedaron marcados "Tentativo — sujeto a ajustes" (2/7/2026). Lección ETC 89: cerrar el presupuesto formalmente antes del retiro y marcar las donaciones en especie al recibirlas.</t>
+          <t>Costo real 5,306.11 asumido por los directores; en la especie se valora a ppto (2,300) por instrucción del director. Solo informativo.</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr"/>
@@ -8032,15 +8074,33 @@
       </c>
       <c r="B25" s="70" t="inlineStr">
         <is>
+          <t>Presupuestos "Tentativo"</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>Ambos quedaron marcados "Tentativo — sujeto a ajustes" (2/7/2026). Lección ETC 89: cerrar el presupuesto formalmente antes del retiro y marcar las donaciones en especie al recibirlas.</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="71" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B26" s="70" t="inlineStr">
+        <is>
           <t>Tablero público</t>
         </is>
       </c>
-      <c r="C25" s="39" t="inlineStr">
+      <c r="C26" s="39" t="inlineStr">
         <is>
           <t>Vista pública: corregido el ancho de las tarjetas y añadida la tarjeta de Profondo (corrección entregada). Falta publicarla.</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>Publicar la corrección en el tablero.</t>
         </is>
@@ -8518,7 +8578,7 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Reembolso. Proforma Paulinas 34,000 + 1,360</t>
+          <t>Reembolso a JM. 52 biblias × 680 = 35,360 exactos. El presupuesto solo tenía 50 (34,000): las 2 de más (1,360) son las que figuraban como 'las pagaría Camila' y terminaron dentro de lo que pagó el grupo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Conciliación: restituida la nota de los 400 sin explicar en las habitaciones
Los 1,800 son firmes (lo que queda del pago a la casa). La tarifa de
900/noche está inferida de ahí, y el desglose verbal del 10-sep
(700 × 2 + 800 = 2,200) daría 400 más de lo que la casa cobró. Queda
como nota: una línea de la factura lo cierra y no afecta ningún total.

Con esto, los tres puntos blandos del cierre quedan visibles en el
documento: el reparto del impuesto, la tarifa de las habitaciones y las
2 biblias de Camila.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016scja59CycFFrqKgYsUPWh
</commit_message>
<xml_diff>
--- a/data/presupuesto/Conciliacion_Final_ETC88.xlsx
+++ b/data/presupuesto/Conciliacion_Final_ETC88.xlsx
@@ -803,7 +803,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3816000" cy="2951999"/>
@@ -825,7 +825,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3816000" cy="2951999"/>
@@ -1136,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1502,7 +1502,7 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>PENDIENTES (0 abiertos · 2 notas)</t>
+          <t>PENDIENTES (0 abiertos · 3 notas)</t>
         </is>
       </c>
     </row>
@@ -1530,142 +1530,154 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Habitaciones de pequeños grupos: 400 sin explicar</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Una línea de la factura de la casa lo cierra. No afecta ningún total: lo pagado es lo pagado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>DISTRIBUCIÓN DEL DINERO</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Izquierda: de dónde salió cada peso que entró. Derecha: en qué se fue cada peso que salió de caja.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="14" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>HOJAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="15" t="inlineStr">
-        <is>
-          <t>1 Caja</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>entradas por fuente, salidas, balance, banco</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>2 Presupuesto vs costo</t>
+          <t>1 Caja</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>presupuestado → costó → cubierto sin pagar → pagado de caja, por área</t>
+          <t>entradas por fuente, salidas, balance, banco</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="inlineStr">
         <is>
-          <t>3 Al costo vs caja</t>
+          <t>2 Presupuesto vs costo</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>qué vale el retiro y qué nos costó; la casa al detalle</t>
+          <t>presupuestado → costó → cubierto sin pagar → pagado de caja, por área</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
         <is>
-          <t>4 Base ETC 89</t>
+          <t>3 Al costo vs caja</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>costo real por partida y por persona; recomendaciones para el próximo</t>
+          <t>qué vale el retiro y qué nos costó; la casa al detalle</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="15" t="inlineStr">
         <is>
-          <t>5 Pendientes</t>
+          <t>4 Base ETC 89</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>una sola lista: abiertos, notas, cerrados</t>
+          <t>costo real por partida y por persona; recomendaciones para el próximo</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="inlineStr">
         <is>
-          <t>6 Ppto oficial vs Sistem</t>
+          <t>5 Pendientes</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>los dos presupuestos por área</t>
+          <t>una sola lista: abiertos, notas, cerrados</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>7–10 Anexos</t>
+          <t>6 Ppto oficial vs Sistem</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Gastos · Donaciones efectivo · Especie · Profondo (con la liquidación de la comisión)</t>
+          <t>los dos presupuestos por área</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>11 Auditoría</t>
+          <t>7–10 Anexos</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>37 verificaciones recalculadas (37 cuadran)</t>
+          <t>Gastos · Donaciones efectivo · Especie · Profondo (con la liquidación de la comisión)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>12 Fuentes y método</t>
+          <t>11 Auditoría</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>de dónde sale cada número y las reglas usadas</t>
+          <t>37 verificaciones recalculadas (37 cuadran)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="15" t="inlineStr">
         <is>
+          <t>12 Fuentes y método</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>de dónde sale cada número y las reglas usadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
           <t>13 Notas por partida</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>la explicación de cada partida del presupuesto</t>
         </is>
@@ -4037,7 +4049,7 @@
       </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
-          <t>Tarifa inferida: 900/noche × 2 noches = 1,800 (240,220 − 228,920 − 9,500)</t>
+          <t>Los 1,800 son firmes: es lo que queda del pago a la casa tras el hospedaje y el jueves (240,220 − 228,920 − 9,500). La tarifa de 900/noche es INFERIDA de ahí. El desglose verbal del 10-sep (700 × 2 noches + 800 de una habitación extra = 2,200) daría 400 más de lo que se pagó: diferencia sin explicar, pendiente de la factura de la casa</t>
         </is>
       </c>
     </row>
@@ -6200,7 +6212,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>tarifa inferida 900/noche</t>
+          <t>monto firme; tarifa inferida 900/noche. El desglose verbal (700 × 2 + 800 = 2,200) daría 400 más</t>
         </is>
       </c>
     </row>
@@ -7623,7 +7635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7807,22 +7819,26 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="69" t="inlineStr">
-        <is>
-          <t>CERRADO</t>
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>NOTA</t>
         </is>
       </c>
       <c r="B11" s="70" t="inlineStr">
         <is>
-          <t>Impresión de libretas 1,260</t>
+          <t>Habitaciones de pequeños grupos: 400 sin explicar</t>
         </is>
       </c>
       <c r="C11" s="39" t="inlineStr">
         <is>
-          <t>El presupuesto operativo la marcaba "donado por guías" en la columna equivocada, por eso no sumaba. Sumada a la especie por confirmación del director (11-sep).</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr"/>
+          <t>Los 1,800 son firmes: es lo que queda del pago a la casa tras el hospedaje (228,920) y el jueves (9,500). La tarifa de 900/noche está inferida de ahí. El desglose que dio la dirección el 10-sep (700 × 2 noches + 800 de una habitación extra) suma 2,200, o sea 400 más de lo que la casa cobró.</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Una línea de la factura de la casa lo cierra. No afecta ningún total: lo pagado es lo pagado.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="69" t="inlineStr">
@@ -7832,12 +7848,12 @@
       </c>
       <c r="B12" s="70" t="inlineStr">
         <is>
-          <t>Uso de los 34,337 en cuentas</t>
+          <t>Impresión de libretas 1,260</t>
         </is>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>La dirección lo expondrá en la actividad de cierre (evaluación) del ETC 88 para decidirlo con el equipo (11-sep).</t>
+          <t>El presupuesto operativo la marcaba "donado por guías" en la columna equivocada, por eso no sumaba. Sumada a la especie por confirmación del director (11-sep).</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr"/>
@@ -7850,12 +7866,12 @@
       </c>
       <c r="B13" s="70" t="inlineStr">
         <is>
-          <t>Profondo: liquidación de la comisión</t>
+          <t>Uso de los 34,337 en cuentas</t>
         </is>
       </c>
       <c r="C13" s="39" t="inlineStr">
         <is>
-          <t>Bruto 154,420: 680.5 boletas pagadas × 200 = 136,100 + venta de comida y helados 18,320. Premios 19,900 (aire acondicionado 16,900 + abanico de torre 3,000). Neto del informe 134,520; entregado a finanzas 135,866.40: los 1,346.40 adicionales son ventas de helados posteriores al informe (director).</t>
+          <t>La dirección lo expondrá en la actividad de cierre (evaluación) del ETC 88 para decidirlo con el equipo (11-sep).</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr"/>
@@ -7868,12 +7884,12 @@
       </c>
       <c r="B14" s="70" t="inlineStr">
         <is>
-          <t>Pagaron y no fueron</t>
+          <t>Profondo: liquidación de la comisión</t>
         </is>
       </c>
       <c r="C14" s="39" t="inlineStr">
         <is>
-          <t>Verificado nombre por nombre contra la lista de pagos del director (10-sep, 57 líneas), el registro de cuotas y las 49 donaciones. Equipo: Mary Carmen Ramírez pagó y no asistió; sus 2,000 están dentro de los 98,000. Participantes: los 46 que pagaron están todos identificados con nombre y ninguno figura como ausente. Boris pagó, no fue, se le devolvió una parte y el neto de 1,500 entró como donación a nombre de Jonathan Medina (31/08): su dinero NO está en los 156,800. De Amanda Rivera no hay ningún pago en ninguna fuente; solo aparece en el formulario de junio como invitada de Pamela Colón y Roselyn Quiroz. Los únicos abonos de 500 de la lista son de Melany Ceverino y Erilis Polanco, ambas personas que sí asistieron.</t>
+          <t>Bruto 154,420: 680.5 boletas pagadas × 200 = 136,100 + venta de comida y helados 18,320. Premios 19,900 (aire acondicionado 16,900 + abanico de torre 3,000). Neto del informe 134,520; entregado a finanzas 135,866.40: los 1,346.40 adicionales son ventas de helados posteriores al informe (director).</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr"/>
@@ -7886,12 +7902,12 @@
       </c>
       <c r="B15" s="70" t="inlineStr">
         <is>
-          <t>Presupuesto oficial</t>
+          <t>Pagaron y no fueron</t>
         </is>
       </c>
       <c r="C15" s="39" t="inlineStr">
         <is>
-          <t>Declarado OFICIAL el de 11-Ago (596,249.56, costo completo, tarifa real de la casa). El Sistem (512,859.56) es la referencia operativa del tablero.</t>
+          <t>Verificado nombre por nombre contra la lista de pagos del director (10-sep, 57 líneas), el registro de cuotas y las 49 donaciones. Equipo: Mary Carmen Ramírez pagó y no asistió; sus 2,000 están dentro de los 98,000. Participantes: los 46 que pagaron están todos identificados con nombre y ninguno figura como ausente. Boris pagó, no fue, se le devolvió una parte y el neto de 1,500 entró como donación a nombre de Jonathan Medina (31/08): su dinero NO está en los 156,800. De Amanda Rivera no hay ningún pago en ninguna fuente; solo aparece en el formulario de junio como invitada de Pamela Colón y Roselyn Quiroz. Los únicos abonos de 500 de la lista son de Melany Ceverino y Erilis Polanco, ambas personas que sí asistieron.</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr"/>
@@ -7904,19 +7920,15 @@
       </c>
       <c r="B16" s="70" t="inlineStr">
         <is>
-          <t>Pago a JM 37,500</t>
+          <t>Presupuesto oficial</t>
         </is>
       </c>
       <c r="C16" s="39" t="inlineStr">
         <is>
-          <t>Desglosado en la hoja de Gastos: transporte 2ª mitad 17,500 (10,000 + 7,500) + desvío 10,000 + ofrenda P. Héctor 10,000.</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Registrar el desglose en el tablero.</t>
-        </is>
-      </c>
+          <t>Declarado OFICIAL el de 11-Ago (596,249.56, costo completo, tarifa real de la casa). El Sistem (512,859.56) es la referencia operativa del tablero.</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="69" t="inlineStr">
@@ -7926,15 +7938,19 @@
       </c>
       <c r="B17" s="70" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Pago a JM 37,500</t>
         </is>
       </c>
       <c r="C17" s="39" t="inlineStr">
         <is>
-          <t>Fuimos 99, facturadas 97. Cortesías: el padre y la sor (la del director cedida a la sor). Jueves: 27 personas, 19 pagaron 500, 8 sin cobro. Habitaciones de pequeños grupos: 900 × 2 noches. Total 240,220 = avance 23,600 + final 216,620.</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr"/>
+          <t>Desglosado en la hoja de Gastos: transporte 2ª mitad 17,500 (10,000 + 7,500) + desvío 10,000 + ofrenda P. Héctor 10,000.</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Registrar el desglose en el tablero.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="69" t="inlineStr">
@@ -7944,12 +7960,12 @@
       </c>
       <c r="B18" s="70" t="inlineStr">
         <is>
-          <t>Bizcocho y helados</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="C18" s="39" t="inlineStr">
         <is>
-          <t>Bizcocho de bienvenida 6,000 (10/09, no presupuestado). El bizcocho de la dinámica (ppto Cocina 1,500) se cambió por helados: 1,740 (07/09). La venta de helados del profondo es ingreso, no costo.</t>
+          <t>Fuimos 99, facturadas 97. Cortesías: el padre y la sor (la del director cedida a la sor). Jueves: 27 personas, 19 pagaron 500, 8 sin cobro. Habitaciones de pequeños grupos: 900 × 2 noches. Total 240,220 = avance 23,600 + final 216,620.</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr"/>
@@ -7962,12 +7978,12 @@
       </c>
       <c r="B19" s="70" t="inlineStr">
         <is>
-          <t>Lapiceros e insumos de misa</t>
+          <t>Bizcocho y helados</t>
         </is>
       </c>
       <c r="C19" s="39" t="inlineStr">
         <is>
-          <t>Caja de lapiceros (650) donada; insumos de misa (3,000) asumidos por Jonathan Medina y Fernando Cordero. Ambos en la especie.</t>
+          <t>Bizcocho de bienvenida 6,000 (10/09, no presupuestado). El bizcocho de la dinámica (ppto Cocina 1,500) se cambió por helados: 1,740 (07/09). La venta de helados del profondo es ingreso, no costo.</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr"/>
@@ -7980,12 +7996,12 @@
       </c>
       <c r="B20" s="70" t="inlineStr">
         <is>
-          <t>Impresiones de guías</t>
+          <t>Lapiceros e insumos de misa</t>
         </is>
       </c>
       <c r="C20" s="39" t="inlineStr">
         <is>
-          <t>Mochilas (3,600, pagadas) e "impresiones diversas" (3,600, donadas por Darianny) son trabajos distintos. No hay doble conteo.</t>
+          <t>Caja de lapiceros (650) donada; insumos de misa (3,000) asumidos por Jonathan Medina y Fernando Cordero. Ambos en la especie.</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr"/>
@@ -7998,12 +8014,12 @@
       </c>
       <c r="B21" s="70" t="inlineStr">
         <is>
-          <t>Priscila</t>
+          <t>Impresiones de guías</t>
         </is>
       </c>
       <c r="C21" s="39" t="inlineStr">
         <is>
-          <t>Donó materiales (7,340) y recibió 2,000 en efectivo (21/07). Donación neta 5,340; la especie ya lo descuenta.</t>
+          <t>Mochilas (3,600, pagadas) e "impresiones diversas" (3,600, donadas por Darianny) son trabajos distintos. No hay doble conteo.</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr"/>
@@ -8016,37 +8032,37 @@
       </c>
       <c r="B22" s="70" t="inlineStr">
         <is>
+          <t>Priscila</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>Donó materiales (7,340) y recibió 2,000 en efectivo (21/07). Donación neta 5,340; la especie ya lo descuenta.</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="69" t="inlineStr">
+        <is>
+          <t>CERRADO</t>
+        </is>
+      </c>
+      <c r="B23" s="70" t="inlineStr">
+        <is>
           <t>Balance 117,611 de la hoja General</t>
         </is>
       </c>
-      <c r="C22" s="39" t="inlineStr">
+      <c r="C23" s="39" t="inlineStr">
         <is>
           <t>Cifra escrita a mano hacia el 11-ago, antes del retiro. No es un segundo balance. El oficial es 36,543.40 → real 34,337.</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>Borrar o anotar esa cifra en la hoja de presupuesto.</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="71" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="B23" s="70" t="inlineStr">
-        <is>
-          <t>Especie</t>
-        </is>
-      </c>
-      <c r="C23" s="39" t="inlineStr">
-        <is>
-          <t>Total 92,405: la hoja de presupuesto solo tenía marcados 30,301 (marcas sin actualizar). Peces (36,000), decoración (10,300), Bono Olé (4,588), insumos de misa (3,000), oficina, lapiceros y cocina no estaban marcados.</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="71" t="inlineStr">
@@ -8056,12 +8072,12 @@
       </c>
       <c r="B24" s="70" t="inlineStr">
         <is>
-          <t>Oficina</t>
+          <t>Especie</t>
         </is>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
-          <t>Costo real 5,306.11 asumido por los directores; en la especie se valora a ppto (2,300) por instrucción del director. Solo informativo.</t>
+          <t>Total 92,405: la hoja de presupuesto solo tenía marcados 30,301 (marcas sin actualizar). Peces (36,000), decoración (10,300), Bono Olé (4,588), insumos de misa (3,000), oficina, lapiceros y cocina no estaban marcados.</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr"/>
@@ -8074,12 +8090,12 @@
       </c>
       <c r="B25" s="70" t="inlineStr">
         <is>
-          <t>Presupuestos "Tentativo"</t>
+          <t>Oficina</t>
         </is>
       </c>
       <c r="C25" s="39" t="inlineStr">
         <is>
-          <t>Ambos quedaron marcados "Tentativo — sujeto a ajustes" (2/7/2026). Lección ETC 89: cerrar el presupuesto formalmente antes del retiro y marcar las donaciones en especie al recibirlas.</t>
+          <t>Costo real 5,306.11 asumido por los directores; en la especie se valora a ppto (2,300) por instrucción del director. Solo informativo.</t>
         </is>
       </c>
       <c r="D25" s="18" t="inlineStr"/>
@@ -8092,15 +8108,33 @@
       </c>
       <c r="B26" s="70" t="inlineStr">
         <is>
+          <t>Presupuestos "Tentativo"</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>Ambos quedaron marcados "Tentativo — sujeto a ajustes" (2/7/2026). Lección ETC 89: cerrar el presupuesto formalmente antes del retiro y marcar las donaciones en especie al recibirlas.</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="71" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B27" s="70" t="inlineStr">
+        <is>
           <t>Tablero público</t>
         </is>
       </c>
-      <c r="C26" s="39" t="inlineStr">
+      <c r="C27" s="39" t="inlineStr">
         <is>
           <t>Vista pública: corregido el ancho de las tarjetas y añadida la tarjeta de Profondo (corrección entregada). Falta publicarla.</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>Publicar la corrección en el tablero.</t>
         </is>

</xml_diff>